<commit_message>
Additional model reduction examples, corrected construction of matrices for H2 model reduction in h2sisored3.m and h2sisored3_discrete.m
</commit_message>
<xml_diff>
--- a/Comparison_ARMA.xlsx
+++ b/Comparison_ARMA.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\MEP\RMEP_homotopy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B606C1-51F9-46A5-81A5-8FEBECD31D81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EDD9A4F-B719-4B1C-90E9-4480CDBBFB17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25776" yWindow="348" windowWidth="19908" windowHeight="17028" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1380" yWindow="828" windowWidth="21516" windowHeight="17028" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ARMA(1,1)" sheetId="1" r:id="rId1"/>
+    <sheet name="ARMA(2,1)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="38">
   <si>
     <t>n</t>
   </si>
@@ -122,9 +123,6 @@
     <t>3,8GB</t>
   </si>
   <si>
-    <t>homotopy (GPU)</t>
-  </si>
-  <si>
     <t>homotopy new</t>
   </si>
   <si>
@@ -132,6 +130,27 @@
   </si>
   <si>
     <t>Razmerje</t>
+  </si>
+  <si>
+    <t>homotopy</t>
+  </si>
+  <si>
+    <t>paths</t>
+  </si>
+  <si>
+    <t>run1</t>
+  </si>
+  <si>
+    <t>run2</t>
+  </si>
+  <si>
+    <t>run3</t>
+  </si>
+  <si>
+    <t>homotopy (last)</t>
+  </si>
+  <si>
+    <t>razmerje</t>
   </si>
 </sst>
 </file>
@@ -143,7 +162,7 @@
     <numFmt numFmtId="164" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -158,8 +177,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -190,6 +217,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -204,7 +237,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -213,6 +246,15 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="43" fontId="0" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -494,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE34"/>
+  <dimension ref="A1:AE42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.33203125" customWidth="1"/>
@@ -532,10 +574,10 @@
         <v>9</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>15</v>
@@ -556,13 +598,13 @@
         <v>25</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>24</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>15</v>
@@ -612,21 +654,21 @@
         <v>1.0988</v>
       </c>
       <c r="F2" s="4"/>
-      <c r="G2" s="7">
-        <v>0.57330000000000003</v>
+      <c r="G2" s="8">
+        <v>0.7389</v>
       </c>
       <c r="K2" s="5">
         <v>7.8178999999999992E-3</v>
       </c>
-      <c r="N2" s="7">
+      <c r="N2" s="8">
         <v>5.6540000000000002E-3</v>
       </c>
       <c r="P2" s="5">
         <f>G2/N2</f>
-        <v>101.39724089140432</v>
+        <v>130.68623983020871</v>
       </c>
       <c r="T2" s="6">
-        <v>0.45184000000000002</v>
+        <v>0.40899999999999997</v>
       </c>
       <c r="AD2" s="2">
         <f t="shared" ref="AD2:AD8" si="0">E2/K2</f>
@@ -655,7 +697,7 @@
         <v>1.3233E-2</v>
       </c>
       <c r="T3" s="6">
-        <v>2.58</v>
+        <v>2.2189000000000001</v>
       </c>
       <c r="AD3" s="2">
         <f t="shared" si="0"/>
@@ -679,8 +721,8 @@
         <v>3.5832999999999999</v>
       </c>
       <c r="F4" s="4"/>
-      <c r="G4" s="7">
-        <v>1.659</v>
+      <c r="G4" s="8">
+        <v>1.3524</v>
       </c>
       <c r="H4" s="1">
         <v>1.3E-14</v>
@@ -694,12 +736,12 @@
       <c r="K4" s="5">
         <v>2.5798999999999999E-2</v>
       </c>
-      <c r="N4" s="7">
-        <v>1.6330000000000001E-2</v>
+      <c r="N4" s="8">
+        <v>1.36288E-2</v>
       </c>
       <c r="P4" s="5">
         <f>G4/N4</f>
-        <v>101.59216166564605</v>
+        <v>99.231040150270019</v>
       </c>
       <c r="Q4" s="1">
         <v>3.3000000000000002E-9</v>
@@ -711,7 +753,7 @@
         <v>5.7999999999999996E-16</v>
       </c>
       <c r="T4" s="6">
-        <v>8.4389000000000003</v>
+        <v>7.5732999999999997</v>
       </c>
       <c r="U4" s="1">
         <v>1.2E-2</v>
@@ -767,7 +809,7 @@
         <v>2.1999999999999999E-15</v>
       </c>
       <c r="T5" s="6">
-        <v>32.259</v>
+        <v>42.113700000000001</v>
       </c>
       <c r="U5" s="1">
         <v>1.9E-2</v>
@@ -802,8 +844,8 @@
       <c r="F6" s="4">
         <v>6.84</v>
       </c>
-      <c r="G6" s="7">
-        <v>3.0861999999999998</v>
+      <c r="G6" s="8">
+        <v>2.9954499999999999</v>
       </c>
       <c r="H6" s="1">
         <v>5.1999999999999997E-16</v>
@@ -817,12 +859,12 @@
       <c r="K6" s="5">
         <v>9.3600000000000003E-2</v>
       </c>
-      <c r="N6" s="7">
-        <v>3.1649999999999998E-2</v>
+      <c r="N6" s="8">
+        <v>3.0044999999999999E-2</v>
       </c>
       <c r="P6" s="5">
         <f>G6/N6</f>
-        <v>97.510268562401265</v>
+        <v>99.698785155599936</v>
       </c>
       <c r="Q6" s="1">
         <v>2.6000000000000001E-9</v>
@@ -834,7 +876,7 @@
         <v>1.4000000000000001E-15</v>
       </c>
       <c r="T6" s="6">
-        <v>98.078000000000003</v>
+        <v>98.501999999999995</v>
       </c>
       <c r="U6" s="1">
         <v>1.7000000000000001E-2</v>
@@ -919,8 +961,8 @@
       <c r="F8" s="4">
         <v>12.05</v>
       </c>
-      <c r="G8" s="7">
-        <v>6.57</v>
+      <c r="G8" s="8">
+        <v>6.3002000000000002</v>
       </c>
       <c r="H8" s="1">
         <v>7.6000000000000002E-16</v>
@@ -934,12 +976,12 @@
       <c r="K8" s="5">
         <v>0.25488</v>
       </c>
-      <c r="N8" s="7">
-        <v>5.849E-2</v>
+      <c r="N8" s="8">
+        <v>6.2210000000000001E-2</v>
       </c>
       <c r="P8" s="5">
         <f>G8/N8</f>
-        <v>112.326893486066</v>
+        <v>101.27310721748916</v>
       </c>
       <c r="Q8" s="1">
         <v>3.6E-9</v>
@@ -983,8 +1025,8 @@
         <v>36.363999999999997</v>
       </c>
       <c r="F10" s="4"/>
-      <c r="G10" s="7">
-        <v>12.62</v>
+      <c r="G10" s="8">
+        <v>11.462</v>
       </c>
       <c r="H10" s="1">
         <v>3.4E-15</v>
@@ -998,12 +1040,12 @@
       <c r="K10" s="5">
         <v>0.65869999999999995</v>
       </c>
-      <c r="N10" s="7">
-        <v>0.14299999999999999</v>
+      <c r="N10" s="8">
+        <v>0.15228</v>
       </c>
       <c r="P10" s="5">
         <f>G10/N10</f>
-        <v>88.251748251748253</v>
+        <v>75.269240872077745</v>
       </c>
       <c r="Q10" s="1">
         <v>8.0999999999999997E-9</v>
@@ -1044,8 +1086,8 @@
         <v>62.454999999999998</v>
       </c>
       <c r="F12" s="4"/>
-      <c r="G12" s="7">
-        <v>22.18</v>
+      <c r="G12" s="8">
+        <v>21.009</v>
       </c>
       <c r="H12" s="1">
         <v>4.4E-16</v>
@@ -1059,12 +1101,12 @@
       <c r="K12" s="5">
         <v>1.5642</v>
       </c>
-      <c r="N12" s="7">
-        <v>0.28599999999999998</v>
+      <c r="N12" s="8">
+        <v>0.27450000000000002</v>
       </c>
       <c r="P12" s="5">
         <f>G12/N12</f>
-        <v>77.55244755244756</v>
+        <v>76.535519125683052</v>
       </c>
       <c r="Q12" s="1">
         <v>9.8999999999999993E-9</v>
@@ -1121,8 +1163,8 @@
       <c r="F14" s="4">
         <v>70.3</v>
       </c>
-      <c r="G14" s="7">
-        <v>37.659999999999997</v>
+      <c r="G14" s="8">
+        <v>35.284999999999997</v>
       </c>
       <c r="H14" s="1">
         <v>6.2999999999999998E-16</v>
@@ -1136,12 +1178,12 @@
       <c r="K14" s="5">
         <v>3.7884000000000002</v>
       </c>
-      <c r="N14" s="7">
-        <v>0.77800000000000002</v>
+      <c r="N14" s="8">
+        <v>0.71489999999999998</v>
       </c>
       <c r="P14" s="5">
         <f>G14/N14</f>
-        <v>48.406169665809763</v>
+        <v>49.356553364106865</v>
       </c>
       <c r="Q14" s="1">
         <v>1.8E-9</v>
@@ -1181,8 +1223,8 @@
       <c r="F16" s="4">
         <v>132.77699999999999</v>
       </c>
-      <c r="G16" s="7">
-        <v>59.49</v>
+      <c r="G16" s="8">
+        <v>55.04</v>
       </c>
       <c r="K16" s="5">
         <v>8.1417999999999999</v>
@@ -1193,12 +1235,12 @@
       <c r="M16" s="5">
         <v>4.6399999999999997</v>
       </c>
-      <c r="N16" s="7">
-        <v>1.4410000000000001</v>
+      <c r="N16" s="8">
+        <v>1.48</v>
       </c>
       <c r="P16" s="5">
         <f>G16/N16</f>
-        <v>41.283830673143648</v>
+        <v>37.189189189189186</v>
       </c>
       <c r="AD16" s="2">
         <f>E16/K16</f>
@@ -1226,8 +1268,8 @@
       <c r="F18" s="4">
         <v>198.7</v>
       </c>
-      <c r="G18" s="7">
-        <v>81.7</v>
+      <c r="G18" s="8">
+        <v>72.686000000000007</v>
       </c>
       <c r="K18" s="5">
         <v>15.597</v>
@@ -1238,12 +1280,12 @@
       <c r="M18" s="5">
         <v>8.94</v>
       </c>
-      <c r="N18" s="7">
-        <v>2.9769999999999999</v>
+      <c r="N18" s="8">
+        <v>2.89</v>
       </c>
       <c r="P18" s="5">
         <f>G18/N18</f>
-        <v>27.443735303997315</v>
+        <v>25.150865051903114</v>
       </c>
       <c r="AD18" s="2">
         <f>E18/K18</f>
@@ -1269,8 +1311,8 @@
         <v>382.46</v>
       </c>
       <c r="F20" s="4"/>
-      <c r="G20" s="7">
-        <v>124.39</v>
+      <c r="G20" s="8">
+        <v>108.015</v>
       </c>
       <c r="K20" s="5">
         <v>24.78</v>
@@ -1281,12 +1323,12 @@
       <c r="M20" s="5">
         <v>9.9700000000000006</v>
       </c>
-      <c r="N20" s="7">
-        <v>5.4809999999999999</v>
+      <c r="N20" s="8">
+        <v>5.4</v>
       </c>
       <c r="P20" s="5">
         <f>G20/N20</f>
-        <v>22.694763729246489</v>
+        <v>20.002777777777776</v>
       </c>
       <c r="AD20" s="2">
         <f>E20/K20</f>
@@ -1312,12 +1354,21 @@
         <v>519.46</v>
       </c>
       <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="G22" s="8">
+        <v>149.54560000000001</v>
+      </c>
       <c r="K22" s="5">
         <v>40.44</v>
       </c>
       <c r="L22" s="5">
         <v>28.08</v>
+      </c>
+      <c r="N22" s="8">
+        <v>9.14</v>
+      </c>
+      <c r="P22" s="5">
+        <f>G22/N22</f>
+        <v>16.361663019693655</v>
       </c>
       <c r="AD22" s="2">
         <f>E22/K22</f>
@@ -1343,7 +1394,9 @@
         <v>768.79</v>
       </c>
       <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
+      <c r="G24" s="8">
+        <v>205.61699999999999</v>
+      </c>
       <c r="K24" s="5">
         <v>64.594999999999999</v>
       </c>
@@ -1353,8 +1406,12 @@
       <c r="M24" s="5">
         <v>24.92</v>
       </c>
-      <c r="N24" s="5">
-        <v>17.84</v>
+      <c r="N24" s="8">
+        <v>15.134</v>
+      </c>
+      <c r="P24" s="5">
+        <f>G24/N24</f>
+        <v>13.586427910664728</v>
       </c>
       <c r="AD24" s="2">
         <f>E24/K24</f>
@@ -1380,8 +1437,8 @@
         <v>1081.4000000000001</v>
       </c>
       <c r="F26" s="4"/>
-      <c r="G26" s="4">
-        <v>679</v>
+      <c r="G26" s="8">
+        <v>276.83359999999999</v>
       </c>
       <c r="K26" s="5">
         <v>97.626999999999995</v>
@@ -1392,8 +1449,12 @@
       <c r="M26" s="5">
         <v>33.18</v>
       </c>
-      <c r="N26" s="5">
-        <v>24.75</v>
+      <c r="N26" s="8">
+        <v>24.049199999999999</v>
+      </c>
+      <c r="P26" s="5">
+        <f>G26/N26</f>
+        <v>11.511135505546962</v>
       </c>
       <c r="AD26" s="2">
         <f>E26/K26</f>
@@ -1421,8 +1482,8 @@
       <c r="F28" s="4">
         <v>1246.5999999999999</v>
       </c>
-      <c r="G28" s="7">
-        <v>535.11</v>
+      <c r="G28" s="8">
+        <v>367.87900000000002</v>
       </c>
       <c r="K28" s="5">
         <v>139.9</v>
@@ -1433,12 +1494,12 @@
       <c r="M28" s="5">
         <v>53.34</v>
       </c>
-      <c r="N28" s="5">
-        <v>39.19</v>
+      <c r="N28" s="8">
+        <v>37.215000000000003</v>
       </c>
       <c r="P28" s="5">
         <f>G28/N28</f>
-        <v>13.654248532788978</v>
+        <v>9.8852344484750763</v>
       </c>
       <c r="AD28" s="2">
         <f>E28/K28</f>
@@ -1447,85 +1508,553 @@
     </row>
     <row r="30" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B30">
-        <v>469</v>
+        <v>427</v>
       </c>
       <c r="D30">
-        <v>10712</v>
-      </c>
-      <c r="E30" s="3">
-        <v>2899</v>
-      </c>
-      <c r="G30" s="3">
-        <v>2267</v>
-      </c>
-      <c r="H30" s="1">
-        <v>2E-16</v>
-      </c>
-      <c r="I30" s="1">
-        <v>1.8E-17</v>
-      </c>
-      <c r="J30" s="1">
-        <v>3.0999999999999998E-17</v>
-      </c>
-      <c r="K30" s="5">
-        <v>339.95</v>
-      </c>
-      <c r="L30" s="5">
-        <v>235.36</v>
-      </c>
-      <c r="M30" s="5">
-        <v>120.98</v>
-      </c>
-      <c r="N30" s="7">
-        <v>96.65</v>
-      </c>
-      <c r="O30" s="5" t="s">
-        <v>26</v>
+        <v>8918</v>
+      </c>
+      <c r="G30" s="9">
+        <v>569.78859999999997</v>
+      </c>
+      <c r="N30" s="8">
+        <v>53.883000000000003</v>
       </c>
       <c r="P30" s="5">
         <f>G30/N30</f>
-        <v>23.455768235902742</v>
-      </c>
-      <c r="Q30" s="1">
-        <v>1.6000000000000001E-9</v>
-      </c>
-      <c r="R30" s="1">
-        <v>9.2000000000000005E-11</v>
-      </c>
-      <c r="S30" s="1">
-        <v>6.6E-15</v>
-      </c>
-      <c r="AD30" s="2">
-        <f>E30/K30</f>
-        <v>8.52772466539197</v>
+        <v>10.574552270660504</v>
       </c>
     </row>
     <row r="32" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A32">
+        <v>34</v>
+      </c>
+      <c r="B32">
+        <v>455</v>
+      </c>
+      <c r="D32">
+        <v>10100</v>
+      </c>
+      <c r="G32" s="9">
+        <v>776.55830000000003</v>
+      </c>
+      <c r="N32" s="8">
+        <v>78.072999999999993</v>
+      </c>
+      <c r="P32" s="5">
+        <f>G32/N32</f>
+        <v>9.9465666747787331</v>
+      </c>
+    </row>
+    <row r="33" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>35</v>
+      </c>
+      <c r="B33">
+        <v>469</v>
+      </c>
+      <c r="D33">
+        <v>10712</v>
+      </c>
+      <c r="E33" s="3">
+        <v>2899</v>
+      </c>
+      <c r="G33" s="3">
+        <v>2267</v>
+      </c>
+      <c r="H33" s="1">
+        <v>2E-16</v>
+      </c>
+      <c r="I33" s="1">
+        <v>1.8E-17</v>
+      </c>
+      <c r="J33" s="1">
+        <v>3.0999999999999998E-17</v>
+      </c>
+      <c r="K33" s="5">
+        <v>339.95</v>
+      </c>
+      <c r="L33" s="5">
+        <v>235.36</v>
+      </c>
+      <c r="M33" s="5">
+        <v>120.98</v>
+      </c>
+      <c r="N33" s="7">
+        <v>96.65</v>
+      </c>
+      <c r="O33" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="P33" s="5">
+        <f>G33/N33</f>
+        <v>23.455768235902742</v>
+      </c>
+      <c r="Q33" s="1">
+        <v>1.6000000000000001E-9</v>
+      </c>
+      <c r="R33" s="1">
+        <v>9.2000000000000005E-11</v>
+      </c>
+      <c r="S33" s="1">
+        <v>6.6E-15</v>
+      </c>
+      <c r="AD33" s="2">
+        <f>E33/K33</f>
+        <v>8.52772466539197</v>
+      </c>
+    </row>
+    <row r="36" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>40</v>
+      </c>
+      <c r="B36">
+        <v>539</v>
+      </c>
+      <c r="D36">
+        <v>14042</v>
+      </c>
+      <c r="G36" s="9">
+        <v>2429.2469999999998</v>
+      </c>
+      <c r="N36" s="8">
+        <v>209.85579999999999</v>
+      </c>
+      <c r="P36" s="5">
+        <f>G36/N36</f>
+        <v>11.575791567352439</v>
+      </c>
+    </row>
+    <row r="38" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>45</v>
+      </c>
+      <c r="B38">
+        <v>609</v>
+      </c>
+      <c r="D38">
+        <v>17822</v>
+      </c>
+      <c r="G38" s="9">
+        <v>4890.5200000000004</v>
+      </c>
+      <c r="N38" s="8">
+        <v>427.77</v>
+      </c>
+      <c r="P38" s="5">
+        <f>G38/N38</f>
+        <v>11.432592280898616</v>
+      </c>
+    </row>
+    <row r="40" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A40">
         <v>50</v>
       </c>
-      <c r="D32">
+      <c r="D40">
         <v>22052</v>
       </c>
-      <c r="M32" s="5">
+      <c r="M40" s="5">
         <v>921.11</v>
       </c>
-      <c r="N32" s="7">
+      <c r="N40" s="7">
         <v>825.24</v>
       </c>
-      <c r="O32" s="5" t="s">
+      <c r="O40" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34">
+    <row r="42" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A42">
         <v>60</v>
       </c>
-      <c r="D34">
+      <c r="D42">
         <v>31862</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51572A20-BB7E-44BE-B5FD-2A26A68D3982}">
+  <dimension ref="A1:K12"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.77734375" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.44140625" style="10" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" s="15" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="15">
+        <v>5</v>
+      </c>
+      <c r="B2" s="15">
+        <v>13</v>
+      </c>
+      <c r="C2" s="15">
+        <v>3</v>
+      </c>
+      <c r="D2" s="15">
+        <v>3</v>
+      </c>
+      <c r="E2" s="15">
+        <v>0</v>
+      </c>
+      <c r="F2" s="15">
+        <v>910</v>
+      </c>
+      <c r="G2" s="16">
+        <v>5.1694000000000004</v>
+      </c>
+      <c r="H2" s="16">
+        <v>0.10299999999999999</v>
+      </c>
+      <c r="K2" s="10">
+        <f t="shared" ref="K2:K12" si="0">G2/H2</f>
+        <v>50.188349514563114</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>6</v>
+      </c>
+      <c r="B3">
+        <v>21</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>1938</v>
+      </c>
+      <c r="G3" s="10">
+        <v>12.374000000000001</v>
+      </c>
+      <c r="H3" s="10">
+        <v>0.43109999999999998</v>
+      </c>
+      <c r="K3" s="10">
+        <f t="shared" si="0"/>
+        <v>28.703317095801442</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>29</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>3542</v>
+      </c>
+      <c r="G4" s="10">
+        <v>25.800999999999998</v>
+      </c>
+      <c r="H4" s="10">
+        <v>1.5449999999999999</v>
+      </c>
+      <c r="K4" s="10">
+        <f t="shared" si="0"/>
+        <v>16.699676375404529</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>47</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>5850</v>
+      </c>
+      <c r="G5" s="10">
+        <v>50.484000000000002</v>
+      </c>
+      <c r="H5" s="10">
+        <v>5.9688999999999997</v>
+      </c>
+      <c r="K5" s="10">
+        <f t="shared" si="0"/>
+        <v>8.4578398029787749</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>45</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>8990</v>
+      </c>
+      <c r="G6" s="10">
+        <v>90.779499999999999</v>
+      </c>
+      <c r="H6" s="10">
+        <v>18.725999999999999</v>
+      </c>
+      <c r="K6" s="10">
+        <f t="shared" si="0"/>
+        <v>4.8477784898002776</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>53</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>13090</v>
+      </c>
+      <c r="G7" s="10">
+        <v>161.54480000000001</v>
+      </c>
+      <c r="H7" s="10">
+        <v>46.996000000000002</v>
+      </c>
+      <c r="K7" s="10">
+        <f t="shared" si="0"/>
+        <v>3.4374159502936421</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>11</v>
+      </c>
+      <c r="B8">
+        <v>61</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>18278</v>
+      </c>
+      <c r="G8" s="10">
+        <v>263.76499999999999</v>
+      </c>
+      <c r="H8" s="10">
+        <v>112.616</v>
+      </c>
+      <c r="K8" s="10">
+        <f t="shared" si="0"/>
+        <v>2.3421627477445477</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>12</v>
+      </c>
+      <c r="B9">
+        <v>69</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>24862</v>
+      </c>
+      <c r="G9" s="10">
+        <v>411.40300000000002</v>
+      </c>
+      <c r="H9" s="10">
+        <v>235.92099999999999</v>
+      </c>
+      <c r="K9" s="10">
+        <f t="shared" si="0"/>
+        <v>1.7438167861275597</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>13</v>
+      </c>
+      <c r="B10">
+        <v>77</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>32430</v>
+      </c>
+      <c r="G10" s="10">
+        <v>634.18359999999996</v>
+      </c>
+      <c r="H10" s="10">
+        <v>473.54399999999998</v>
+      </c>
+      <c r="K10" s="10">
+        <f t="shared" si="0"/>
+        <v>1.3392284560674403</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>14</v>
+      </c>
+      <c r="B11">
+        <v>85</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>41650</v>
+      </c>
+      <c r="G11" s="10">
+        <v>1136.5899999999999</v>
+      </c>
+      <c r="H11" s="10">
+        <v>986.88</v>
+      </c>
+      <c r="K11" s="10">
+        <f t="shared" si="0"/>
+        <v>1.1517003080415045</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>15</v>
+      </c>
+      <c r="B12" s="13">
+        <v>93</v>
+      </c>
+      <c r="C12" s="13">
+        <v>1</v>
+      </c>
+      <c r="D12" s="13">
+        <v>1</v>
+      </c>
+      <c r="E12" s="13">
+        <v>0</v>
+      </c>
+      <c r="F12" s="13">
+        <v>52470</v>
+      </c>
+      <c r="G12" s="14">
+        <v>1451.06</v>
+      </c>
+      <c r="H12" s="14">
+        <v>1762.43</v>
+      </c>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="14">
+        <f t="shared" si="0"/>
+        <v>0.82332915349829494</v>
       </c>
     </row>
   </sheetData>

</xml_diff>